<commit_message>
📊 Horarios actualizados Línea 141 - 3463
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-06-28.xlsx
+++ b/data/horarios-141-2026-06-28.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 01:52:27</t>
+          <t>Última actualización: 05:14:58</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 2</t>
+          <t>Total filas: 15</t>
         </is>
       </c>
     </row>
@@ -473,21 +473,21 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>01:52:27</t>
+          <t>05:14:58</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>03:02</t>
+          <t>05:16</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>70</v>
+        <v>2</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -498,12 +498,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>01:52:27</t>
+          <t>05:14:58</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>03:48</t>
+          <t>05:17</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -512,9 +512,334 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>116</v>
+        <v>3</v>
       </c>
       <c r="E7" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>05:14:58</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>05:21</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>7</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>05:14:58</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>05:46</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>32</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>05:14:58</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>06:00</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>46</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>05:14:58</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>06:08</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>54</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>05:14:58</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>06:12</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>58</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>05:14:58</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>06:29</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>75</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>05:14:58</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>06:35</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>81</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>05:14:58</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>06:38</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>225_C ROCA-H SUR</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>84</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>05:14:58</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>06:40</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>86</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>05:14:58</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>06:41</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>87</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>05:14:58</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>06:58</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>104</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>05:14:58</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>07:02</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>108</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>05:14:58</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>07:13</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>119</v>
+      </c>
+      <c r="E20" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -531,7 +856,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A3"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -544,14 +869,91 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 01:52:27</t>
+          <t>Última actualización: 05:14:58</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 0</t>
+          <t>Total filas: 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Hora_Scrap</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Hora_Llegada</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Linea</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Minutos</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Parada</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>05:14:58</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>06:12</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>58</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>05:14:58</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>07:02</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>108</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>LP1912</t>
         </is>
       </c>
     </row>
@@ -579,7 +981,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 01:52:27</t>
+          <t>Última actualización: 05:14:58</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 3464
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-06-28.xlsx
+++ b/data/horarios-141-2026-06-28.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E20"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 05:14:58</t>
+          <t>Última actualización: 07:35:07</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 15</t>
+          <t>Total filas: 17</t>
         </is>
       </c>
     </row>
@@ -473,17 +473,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>05:14:58</t>
+          <t>07:35:07</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>05:16</t>
+          <t>07:37</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -498,21 +498,21 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>05:14:58</t>
+          <t>07:35:07</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>05:17</t>
+          <t>07:44</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -523,21 +523,21 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>05:14:58</t>
+          <t>07:35:07</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>05:21</t>
+          <t>07:52</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>7</v>
+        <v>17</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -548,21 +548,21 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>05:14:58</t>
+          <t>07:35:07</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>05:46</t>
+          <t>08:01</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -573,21 +573,21 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>05:14:58</t>
+          <t>07:35:07</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>06:00</t>
+          <t>08:06</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>46</v>
+        <v>31</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -598,21 +598,21 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>05:14:58</t>
+          <t>07:35:07</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>06:08</t>
+          <t>08:19</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>54</v>
+        <v>44</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -623,21 +623,21 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>05:14:58</t>
+          <t>07:35:07</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>06:12</t>
+          <t>08:21</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>58</v>
+        <v>46</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -648,21 +648,21 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>05:14:58</t>
+          <t>07:35:07</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>06:29</t>
+          <t>08:26</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>75</v>
+        <v>51</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -673,21 +673,21 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>05:14:58</t>
+          <t>07:35:07</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>06:35</t>
+          <t>08:45</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>81</v>
+        <v>70</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -698,21 +698,21 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>05:14:58</t>
+          <t>07:35:07</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>06:38</t>
+          <t>08:45</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>84</v>
+        <v>70</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -723,21 +723,21 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>05:14:58</t>
+          <t>07:35:07</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>06:40</t>
+          <t>09:04</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -748,21 +748,21 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>05:14:58</t>
+          <t>07:35:07</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>06:41</t>
+          <t>09:07</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -773,21 +773,21 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>05:14:58</t>
+          <t>07:35:07</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>06:58</t>
+          <t>09:08</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>104</v>
+        <v>93</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -798,21 +798,21 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>05:14:58</t>
+          <t>07:35:07</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>07:02</t>
+          <t>09:16</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>108</v>
+        <v>101</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -823,23 +823,73 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>05:14:58</t>
+          <t>07:35:07</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>07:13</t>
+          <t>09:17</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D20" t="n">
+        <v>102</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>07:35:07</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>09:24</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>109</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>07:35:07</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>09:34</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
         <v>119</v>
       </c>
-      <c r="E20" t="inlineStr">
+      <c r="E22" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -856,7 +906,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -869,14 +919,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 05:14:58</t>
+          <t>Última actualización: 07:35:07</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 2</t>
+          <t>Total filas: 4</t>
         </is>
       </c>
     </row>
@@ -910,12 +960,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>05:14:58</t>
+          <t>07:35:07</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>06:12</t>
+          <t>07:52</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -924,7 +974,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>58</v>
+        <v>17</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -935,23 +985,73 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>05:14:58</t>
+          <t>07:35:07</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>07:02</t>
+          <t>08:45</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>70</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>07:35:07</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>08:45</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>70</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>07:35:07</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>09:07</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
           <t>215A_EL PATO</t>
         </is>
       </c>
-      <c r="D7" t="n">
-        <v>108</v>
-      </c>
-      <c r="E7" t="inlineStr">
+      <c r="D9" t="n">
+        <v>92</v>
+      </c>
+      <c r="E9" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -968,7 +1068,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A3"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -981,14 +1081,116 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 05:14:58</t>
+          <t>Última actualización: 07:35:07</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 0</t>
+          <t>Total filas: 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Hora_Scrap</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Hora_Llegada</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Linea</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Minutos</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Parada</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>07:35:07</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>07:49</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>14</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>07:35:07</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>08:38</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>63</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>07:35:07</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>09:03</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>88</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 3465
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-06-28.xlsx
+++ b/data/horarios-141-2026-06-28.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:E42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 07:35:07</t>
+          <t>Última actualización: 09:05:55</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 17</t>
+          <t>Total filas: 37</t>
         </is>
       </c>
     </row>
@@ -683,7 +683,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -708,7 +708,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D15" t="n">
@@ -748,21 +748,21 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>07:35:07</t>
+          <t>09:05:55</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>09:07</t>
+          <t>09:05</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>92</v>
+        <v>0</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -773,21 +773,21 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>07:35:07</t>
+          <t>09:05:55</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>09:08</t>
+          <t>09:06</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>93</v>
+        <v>1</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -803,16 +803,16 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>09:16</t>
+          <t>09:07</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>101</v>
+        <v>92</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -828,16 +828,16 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>09:17</t>
+          <t>09:08</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>102</v>
+        <v>93</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -848,21 +848,21 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>07:35:07</t>
+          <t>09:05:55</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>09:24</t>
+          <t>09:11</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>109</v>
+        <v>6</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -873,23 +873,523 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>07:35:07</t>
+          <t>09:05:55</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
+          <t>09:16</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>11</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>09:05:55</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>09:16</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>11</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>07:35:07</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>09:17</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>102</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>09:05:55</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>09:23</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>18</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>07:35:07</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>09:24</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>109</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>07:35:07</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
           <t>09:34</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
+      <c r="C27" t="inlineStr">
         <is>
           <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
-      <c r="D22" t="n">
+      <c r="D27" t="n">
         <v>119</v>
       </c>
-      <c r="E22" t="inlineStr">
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>09:05:55</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>09:35</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>30</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>09:05:55</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>09:44</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>39</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>09:05:55</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>09:51</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>46</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>09:05:55</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>09:54</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>49</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>09:05:55</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>09:58</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>53</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>09:05:55</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>10:03</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>58</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>09:05:55</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>10:07</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>62</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>09:05:55</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>10:15</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>70</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>09:05:55</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>10:24</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>79</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>09:05:55</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>10:33</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>88</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>09:05:55</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>10:34</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>89</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>09:05:55</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>10:43</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>98</v>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>09:05:55</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>10:55</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>81_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>110</v>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>09:05:55</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>10:56</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>111</v>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>09:05:55</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>11:04</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>119</v>
+      </c>
+      <c r="E42" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -906,7 +1406,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -919,14 +1419,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 07:35:07</t>
+          <t>Última actualización: 09:05:55</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 4</t>
+          <t>Total filas: 6</t>
         </is>
       </c>
     </row>
@@ -1035,23 +1535,73 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>07:35:07</t>
+          <t>09:05:55</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
+          <t>09:06</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>07:35:07</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
           <t>09:07</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C10" t="inlineStr">
         <is>
           <t>215A_EL PATO</t>
         </is>
       </c>
-      <c r="D9" t="n">
+      <c r="D10" t="n">
         <v>92</v>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>09:05:55</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>09:54</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>49</v>
+      </c>
+      <c r="E11" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1068,7 +1618,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1081,14 +1631,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 07:35:07</t>
+          <t>Última actualización: 09:05:55</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 3</t>
+          <t>Total filas: 7</t>
         </is>
       </c>
     </row>
@@ -1191,6 +1741,106 @@
       <c r="E8" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>09:05:55</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>09:27</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>22</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>09:05:55</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>10:17</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>72</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>09:05:55</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>10:29</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>84</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>09:05:55</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>10:42</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>97</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 3466
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-06-28.xlsx
+++ b/data/horarios-141-2026-06-28.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E42"/>
+  <dimension ref="A1:E61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 09:05:55</t>
+          <t>Última actualización: 11:09:01</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 37</t>
+          <t>Total filas: 56</t>
         </is>
       </c>
     </row>
@@ -1390,6 +1390,481 @@
         <v>119</v>
       </c>
       <c r="E42" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>11:09:01</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>11:09</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>225_C ROCA-H SUR</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>0</v>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>11:09:01</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>11:15</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>6</v>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>11:09:01</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>11:24</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>15</v>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>11:09:01</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>11:35</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>26</v>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>11:09:01</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>11:36</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>27</v>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>11:09:01</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>11:42</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>33</v>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>11:09:01</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>11:45</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>36</v>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>11:09:01</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>11:54</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D50" t="n">
+        <v>45</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>11:09:01</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>11:55</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
+        <v>46</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>11:09:01</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>12:04</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D52" t="n">
+        <v>55</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>11:09:01</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D53" t="n">
+        <v>66</v>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>11:09:01</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>12:25</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D54" t="n">
+        <v>76</v>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>11:09:01</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>12:30</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D55" t="n">
+        <v>81</v>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>11:09:01</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>12:34</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D56" t="n">
+        <v>85</v>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>11:09:01</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>12:37</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D57" t="n">
+        <v>88</v>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>11:09:01</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>12:44</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D58" t="n">
+        <v>95</v>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>11:09:01</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>12:46</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D59" t="n">
+        <v>97</v>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>11:09:01</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>12:55</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D60" t="n">
+        <v>106</v>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>11:09:01</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>13:05</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D61" t="n">
+        <v>116</v>
+      </c>
+      <c r="E61" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1406,7 +1881,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1419,14 +1894,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 09:05:55</t>
+          <t>Última actualización: 11:09:01</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 6</t>
+          <t>Total filas: 9</t>
         </is>
       </c>
     </row>
@@ -1602,6 +2077,81 @@
         <v>49</v>
       </c>
       <c r="E11" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>11:09:01</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>11:35</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>26</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>11:09:01</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>11:45</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>36</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>11:09:01</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>12:55</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>106</v>
+      </c>
+      <c r="E14" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1618,7 +2168,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1631,14 +2181,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 09:05:55</t>
+          <t>Última actualización: 11:09:01</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 7</t>
+          <t>Total filas: 8</t>
         </is>
       </c>
     </row>
@@ -1841,6 +2391,31 @@
       <c r="E12" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>11:09:01</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>11:23</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>14</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 3467
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-06-28.xlsx
+++ b/data/horarios-141-2026-06-28.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E61"/>
+  <dimension ref="A1:E76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 11:09:01</t>
+          <t>Última actualización: 12:37:19</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 56</t>
+          <t>Total filas: 71</t>
         </is>
       </c>
     </row>
@@ -883,7 +883,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D22" t="n">
@@ -908,7 +908,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D23" t="n">
@@ -1748,7 +1748,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>11:09:01</t>
+          <t>12:37:19</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -1762,7 +1762,7 @@
         </is>
       </c>
       <c r="D57" t="n">
-        <v>88</v>
+        <v>0</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
@@ -1773,7 +1773,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>11:09:01</t>
+          <t>12:37:19</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -1787,7 +1787,7 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>95</v>
+        <v>7</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -1798,7 +1798,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>11:09:01</t>
+          <t>12:37:19</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -1812,7 +1812,7 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>97</v>
+        <v>9</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
@@ -1823,7 +1823,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>11:09:01</t>
+          <t>12:37:19</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -1837,7 +1837,7 @@
         </is>
       </c>
       <c r="D60" t="n">
-        <v>106</v>
+        <v>18</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
@@ -1848,23 +1848,398 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
+          <t>12:37:19</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>13:04</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D61" t="n">
+        <v>27</v>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
           <t>11:09:01</t>
         </is>
       </c>
-      <c r="B61" t="inlineStr">
+      <c r="B62" t="inlineStr">
         <is>
           <t>13:05</t>
         </is>
       </c>
-      <c r="C61" t="inlineStr">
+      <c r="C62" t="inlineStr">
         <is>
           <t>11_ETCHEVERRY</t>
         </is>
       </c>
-      <c r="D61" t="n">
+      <c r="D62" t="n">
         <v>116</v>
       </c>
-      <c r="E61" t="inlineStr">
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>12:37:19</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>13:15</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D63" t="n">
+        <v>38</v>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>12:37:19</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>13:21</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D64" t="n">
+        <v>44</v>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>12:37:19</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>13:24</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D65" t="n">
+        <v>47</v>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>12:37:19</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>13:31</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D66" t="n">
+        <v>54</v>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>12:37:19</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>13:44</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D67" t="n">
+        <v>67</v>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>12:37:19</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>13:55</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D68" t="n">
+        <v>78</v>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>12:37:19</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>13:56</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D69" t="n">
+        <v>79</v>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>12:37:19</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>14:04</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D70" t="n">
+        <v>87</v>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>12:37:19</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>14:11</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D71" t="n">
+        <v>94</v>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>12:37:19</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>14:14</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D72" t="n">
+        <v>97</v>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>12:37:19</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>14:14</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D73" t="n">
+        <v>97</v>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>12:37:19</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>14:17</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D74" t="n">
+        <v>100</v>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>12:37:19</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>14:24</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D75" t="n">
+        <v>107</v>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>12:37:19</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>14:35</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D76" t="n">
+        <v>118</v>
+      </c>
+      <c r="E76" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1881,7 +2256,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1894,14 +2269,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 11:09:01</t>
+          <t>Última actualización: 12:37:19</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 9</t>
+          <t>Total filas: 11</t>
         </is>
       </c>
     </row>
@@ -2135,7 +2510,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>11:09:01</t>
+          <t>12:37:19</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -2149,9 +2524,59 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>106</v>
+        <v>18</v>
       </c>
       <c r="E14" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>12:37:19</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>13:31</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>54</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>12:37:19</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>14:35</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>118</v>
+      </c>
+      <c r="E16" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2168,7 +2593,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2181,14 +2606,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 11:09:01</t>
+          <t>Última actualización: 12:37:19</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 8</t>
+          <t>Total filas: 10</t>
         </is>
       </c>
     </row>
@@ -2416,6 +2841,56 @@
       <c r="E13" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>12:37:19</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>13:23</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>46</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>12:37:19</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>13:50</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>73</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 3468
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-06-28.xlsx
+++ b/data/horarios-141-2026-06-28.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E76"/>
+  <dimension ref="A1:E86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:37:19</t>
+          <t>Última actualización: 13:45:34</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 71</t>
+          <t>Total filas: 81</t>
         </is>
       </c>
     </row>
@@ -683,7 +683,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -708,7 +708,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D15" t="n">
@@ -883,7 +883,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D22" t="n">
@@ -908,7 +908,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D23" t="n">
@@ -2023,21 +2023,21 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>12:37:19</t>
+          <t>13:45:34</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>13:55</t>
+          <t>13:45</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>78</v>
+        <v>0</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -2048,21 +2048,21 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>12:37:19</t>
+          <t>13:45:34</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>13:56</t>
+          <t>13:55</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D69" t="n">
-        <v>79</v>
+        <v>10</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
@@ -2073,21 +2073,21 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>12:37:19</t>
+          <t>13:45:34</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>14:04</t>
+          <t>13:56</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D70" t="n">
-        <v>87</v>
+        <v>11</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
@@ -2098,21 +2098,21 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>12:37:19</t>
+          <t>13:45:34</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>14:11</t>
+          <t>14:04</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D71" t="n">
-        <v>94</v>
+        <v>19</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
@@ -2123,21 +2123,21 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>12:37:19</t>
+          <t>13:45:34</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>14:14</t>
+          <t>14:11</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D72" t="n">
-        <v>97</v>
+        <v>26</v>
       </c>
       <c r="E72" t="inlineStr">
         <is>
@@ -2148,7 +2148,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>12:37:19</t>
+          <t>13:45:34</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -2162,7 +2162,7 @@
         </is>
       </c>
       <c r="D73" t="n">
-        <v>97</v>
+        <v>29</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
@@ -2173,21 +2173,21 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>12:37:19</t>
+          <t>13:45:34</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>14:17</t>
+          <t>14:14</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>100</v>
+        <v>29</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -2198,21 +2198,21 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>12:37:19</t>
+          <t>13:45:34</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>14:24</t>
+          <t>14:16</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D75" t="n">
-        <v>107</v>
+        <v>31</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
@@ -2228,18 +2228,268 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
+          <t>14:17</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D76" t="n">
+        <v>100</v>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>13:45:34</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>14:24</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D77" t="n">
+        <v>39</v>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>13:45:34</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>14:31</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D78" t="n">
+        <v>46</v>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>13:45:34</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
           <t>14:35</t>
         </is>
       </c>
-      <c r="C76" t="inlineStr">
+      <c r="C79" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D76" t="n">
-        <v>118</v>
-      </c>
-      <c r="E76" t="inlineStr">
+      <c r="D79" t="n">
+        <v>50</v>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>13:45:34</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>14:44</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D80" t="n">
+        <v>59</v>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>13:45:34</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>14:55</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D81" t="n">
+        <v>70</v>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>13:45:34</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>15:04</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D82" t="n">
+        <v>79</v>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>13:45:34</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>15:04</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D83" t="n">
+        <v>79</v>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>13:45:34</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>15:15</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D84" t="n">
+        <v>90</v>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>13:45:34</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>15:24</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D85" t="n">
+        <v>99</v>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>13:45:34</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>15:35</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D86" t="n">
+        <v>110</v>
+      </c>
+      <c r="E86" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2256,7 +2506,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:E19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2269,14 +2519,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:37:19</t>
+          <t>Última actualización: 13:45:34</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 11</t>
+          <t>Total filas: 14</t>
         </is>
       </c>
     </row>
@@ -2560,7 +2810,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>12:37:19</t>
+          <t>13:45:34</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -2574,9 +2824,84 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>118</v>
+        <v>50</v>
       </c>
       <c r="E16" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>13:45:34</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>14:55</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>70</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>13:45:34</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>15:04</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>79</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>13:45:34</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>15:35</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>110</v>
+      </c>
+      <c r="E19" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2593,7 +2918,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2606,14 +2931,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:37:19</t>
+          <t>Última actualización: 13:45:34</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 10</t>
+          <t>Total filas: 13</t>
         </is>
       </c>
     </row>
@@ -2872,23 +3197,98 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
+          <t>13:45:34</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>13:46</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>1</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
           <t>12:37:19</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B16" t="inlineStr">
         <is>
           <t>13:50</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="C16" t="inlineStr">
         <is>
           <t>215B_LP-P MOR-1 Y 57</t>
         </is>
       </c>
-      <c r="D15" t="n">
+      <c r="D16" t="n">
         <v>73</v>
       </c>
-      <c r="E15" t="inlineStr">
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>13:45:34</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>14:42</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>57</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>13:45:34</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>15:23</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>98</v>
+      </c>
+      <c r="E18" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 3469
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-06-28.xlsx
+++ b/data/horarios-141-2026-06-28.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E86"/>
+  <dimension ref="A1:E101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:45:34</t>
+          <t>Última actualización: 14:49:46</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 81</t>
+          <t>Total filas: 96</t>
         </is>
       </c>
     </row>
@@ -683,7 +683,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -708,7 +708,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D15" t="n">
@@ -883,7 +883,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D22" t="n">
@@ -908,7 +908,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D23" t="n">
@@ -2158,7 +2158,7 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D73" t="n">
@@ -2183,7 +2183,7 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D74" t="n">
@@ -2348,12 +2348,12 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>13:45:34</t>
+          <t>14:49:46</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>14:55</t>
+          <t>14:54</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -2362,7 +2362,7 @@
         </is>
       </c>
       <c r="D81" t="n">
-        <v>70</v>
+        <v>5</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
@@ -2378,16 +2378,16 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>15:04</t>
+          <t>14:55</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D82" t="n">
-        <v>79</v>
+        <v>70</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
@@ -2398,21 +2398,21 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>13:45:34</t>
+          <t>14:49:46</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>15:04</t>
+          <t>15:01</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D83" t="n">
-        <v>79</v>
+        <v>12</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
@@ -2423,21 +2423,21 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>13:45:34</t>
+          <t>14:49:46</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>15:15</t>
+          <t>15:04</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D84" t="n">
-        <v>90</v>
+        <v>15</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
@@ -2453,16 +2453,16 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>15:24</t>
+          <t>15:04</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D85" t="n">
-        <v>99</v>
+        <v>79</v>
       </c>
       <c r="E85" t="inlineStr">
         <is>
@@ -2473,23 +2473,398 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
+          <t>14:49:46</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>15:06</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D86" t="n">
+        <v>17</v>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>14:49:46</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>15:15</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D87" t="n">
+        <v>26</v>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>14:49:46</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>15:24</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D88" t="n">
+        <v>35</v>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>14:49:46</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>15:34</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D89" t="n">
+        <v>45</v>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
           <t>13:45:34</t>
         </is>
       </c>
-      <c r="B86" t="inlineStr">
+      <c r="B90" t="inlineStr">
         <is>
           <t>15:35</t>
         </is>
       </c>
-      <c r="C86" t="inlineStr">
+      <c r="C90" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D86" t="n">
+      <c r="D90" t="n">
         <v>110</v>
       </c>
-      <c r="E86" t="inlineStr">
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>14:49:46</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>15:41</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D91" t="n">
+        <v>52</v>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>14:49:46</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>15:44</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D92" t="n">
+        <v>55</v>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>14:49:46</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>15:51</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D93" t="n">
+        <v>62</v>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>14:49:46</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>15:55</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D94" t="n">
+        <v>66</v>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>14:49:46</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>15:56</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D95" t="n">
+        <v>67</v>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>14:49:46</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>16:04</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D96" t="n">
+        <v>75</v>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>14:49:46</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>16:14</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D97" t="n">
+        <v>85</v>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>14:49:46</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>16:24</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D98" t="n">
+        <v>95</v>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>14:49:46</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>16:34</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D99" t="n">
+        <v>105</v>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>14:49:46</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>16:35</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>83_ALUAR</t>
+        </is>
+      </c>
+      <c r="D100" t="n">
+        <v>106</v>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>14:49:46</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>16:44</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D101" t="n">
+        <v>115</v>
+      </c>
+      <c r="E101" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2506,7 +2881,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:E21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2519,14 +2894,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:45:34</t>
+          <t>Última actualización: 14:49:46</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 14</t>
+          <t>Total filas: 16</t>
         </is>
       </c>
     </row>
@@ -2835,12 +3210,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>13:45:34</t>
+          <t>14:49:46</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>14:55</t>
+          <t>14:54</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -2849,7 +3224,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>70</v>
+        <v>5</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -2865,16 +3240,16 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>15:04</t>
+          <t>14:55</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>79</v>
+        <v>70</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -2885,23 +3260,73 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
+          <t>14:49:46</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>15:04</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>15</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>14:49:46</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>15:34</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>45</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
           <t>13:45:34</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
+      <c r="B21" t="inlineStr">
         <is>
           <t>15:35</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
+      <c r="C21" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D19" t="n">
+      <c r="D21" t="n">
         <v>110</v>
       </c>
-      <c r="E19" t="inlineStr">
+      <c r="E21" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2918,7 +3343,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2931,14 +3356,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:45:34</t>
+          <t>Última actualización: 14:49:46</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 13</t>
+          <t>Total filas: 16</t>
         </is>
       </c>
     </row>
@@ -3272,23 +3697,98 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
+          <t>14:49:46</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>15:22</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>33</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
           <t>13:45:34</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
+      <c r="B19" t="inlineStr">
         <is>
           <t>15:23</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
+      <c r="C19" t="inlineStr">
         <is>
           <t>215A_LA PLATA</t>
         </is>
       </c>
-      <c r="D18" t="n">
+      <c r="D19" t="n">
         <v>98</v>
       </c>
-      <c r="E18" t="inlineStr">
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>14:49:46</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>16:02</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>73</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>14:49:46</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>16:29</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-40 Y 115</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>100</v>
+      </c>
+      <c r="E21" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 3470
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-06-28.xlsx
+++ b/data/horarios-141-2026-06-28.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E101"/>
+  <dimension ref="A1:E114"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:49:46</t>
+          <t>Última actualización: 15:54:07</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 96</t>
+          <t>Total filas: 109</t>
         </is>
       </c>
     </row>
@@ -683,7 +683,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -708,7 +708,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D15" t="n">
@@ -883,7 +883,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D22" t="n">
@@ -908,7 +908,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D23" t="n">
@@ -2158,7 +2158,7 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D73" t="n">
@@ -2183,7 +2183,7 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D74" t="n">
@@ -2423,7 +2423,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>14:49:46</t>
+          <t>13:45:34</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -2433,11 +2433,11 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D84" t="n">
-        <v>15</v>
+        <v>79</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
@@ -2448,7 +2448,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>13:45:34</t>
+          <t>14:49:46</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -2458,11 +2458,11 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D85" t="n">
-        <v>79</v>
+        <v>15</v>
       </c>
       <c r="E85" t="inlineStr">
         <is>
@@ -2673,7 +2673,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>14:49:46</t>
+          <t>15:54:07</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -2687,7 +2687,7 @@
         </is>
       </c>
       <c r="D94" t="n">
-        <v>66</v>
+        <v>1</v>
       </c>
       <c r="E94" t="inlineStr">
         <is>
@@ -2723,21 +2723,21 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>14:49:46</t>
+          <t>15:54:07</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>16:04</t>
+          <t>15:57</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D96" t="n">
-        <v>75</v>
+        <v>3</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
@@ -2748,21 +2748,21 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>14:49:46</t>
+          <t>15:54:07</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>16:14</t>
+          <t>16:04</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D97" t="n">
-        <v>85</v>
+        <v>10</v>
       </c>
       <c r="E97" t="inlineStr">
         <is>
@@ -2773,21 +2773,21 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>14:49:46</t>
+          <t>15:54:07</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>16:24</t>
+          <t>16:14</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D98" t="n">
-        <v>95</v>
+        <v>20</v>
       </c>
       <c r="E98" t="inlineStr">
         <is>
@@ -2798,21 +2798,21 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>14:49:46</t>
+          <t>15:54:07</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>16:34</t>
+          <t>16:16</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D99" t="n">
-        <v>105</v>
+        <v>22</v>
       </c>
       <c r="E99" t="inlineStr">
         <is>
@@ -2828,16 +2828,16 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>16:35</t>
+          <t>16:24</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>83_ALUAR</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D100" t="n">
-        <v>106</v>
+        <v>95</v>
       </c>
       <c r="E100" t="inlineStr">
         <is>
@@ -2848,23 +2848,348 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>14:49:46</t>
+          <t>15:54:07</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
+          <t>16:25</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D101" t="n">
+        <v>31</v>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>15:54:07</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>16:34</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D102" t="n">
+        <v>40</v>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>15:54:07</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>16:35</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>83_ALUAR</t>
+        </is>
+      </c>
+      <c r="D103" t="n">
+        <v>41</v>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>15:54:07</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>16:41</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D104" t="n">
+        <v>47</v>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>15:54:07</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
           <t>16:44</t>
         </is>
       </c>
-      <c r="C101" t="inlineStr">
+      <c r="C105" t="inlineStr">
         <is>
           <t>225_GOMEZ</t>
         </is>
       </c>
-      <c r="D101" t="n">
-        <v>115</v>
-      </c>
-      <c r="E101" t="inlineStr">
+      <c r="D105" t="n">
+        <v>50</v>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>15:54:07</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>16:51</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D106" t="n">
+        <v>57</v>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>15:54:07</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>16:55</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D107" t="n">
+        <v>61</v>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>15:54:07</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>17:05</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D108" t="n">
+        <v>71</v>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>15:54:07</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>17:15</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D109" t="n">
+        <v>81</v>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>15:54:07</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>17:24</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D110" t="n">
+        <v>90</v>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>15:54:07</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>17:32</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D111" t="n">
+        <v>98</v>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>15:54:07</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>17:35</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D112" t="n">
+        <v>101</v>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>15:54:07</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>17:37</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D113" t="n">
+        <v>103</v>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>15:54:07</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>17:45</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D114" t="n">
+        <v>111</v>
+      </c>
+      <c r="E114" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2881,7 +3206,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:E23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2894,14 +3219,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:49:46</t>
+          <t>Última actualización: 15:54:07</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 16</t>
+          <t>Total filas: 18</t>
         </is>
       </c>
     </row>
@@ -3327,6 +3652,56 @@
         <v>110</v>
       </c>
       <c r="E21" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>15:54:07</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>17:15</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>81</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>15:54:07</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>17:45</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>111</v>
+      </c>
+      <c r="E23" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3343,7 +3718,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:E24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3356,14 +3731,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:49:46</t>
+          <t>Última actualización: 15:54:07</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 16</t>
+          <t>Total filas: 19</t>
         </is>
       </c>
     </row>
@@ -3772,25 +4147,100 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
+          <t>15:54:07</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>16:03</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>9</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
           <t>14:49:46</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
+      <c r="B22" t="inlineStr">
         <is>
           <t>16:29</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
+      <c r="C22" t="inlineStr">
         <is>
           <t>215B_LP-P MOR-40 Y 115</t>
         </is>
       </c>
-      <c r="D21" t="n">
+      <c r="D22" t="n">
         <v>100</v>
       </c>
-      <c r="E21" t="inlineStr">
+      <c r="E22" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>15:54:07</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-40 Y 115</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>36</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>15:54:07</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>17:23</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>89</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 3471
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-06-28.xlsx
+++ b/data/horarios-141-2026-06-28.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E114"/>
+  <dimension ref="A1:E126"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 15:54:07</t>
+          <t>Última actualización: 17:04:15</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 109</t>
+          <t>Total filas: 121</t>
         </is>
       </c>
     </row>
@@ -2158,7 +2158,7 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D73" t="n">
@@ -2183,7 +2183,7 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D74" t="n">
@@ -3023,7 +3023,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>15:54:07</t>
+          <t>17:04:15</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
@@ -3037,7 +3037,7 @@
         </is>
       </c>
       <c r="D108" t="n">
-        <v>71</v>
+        <v>1</v>
       </c>
       <c r="E108" t="inlineStr">
         <is>
@@ -3048,7 +3048,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>15:54:07</t>
+          <t>17:04:15</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -3062,7 +3062,7 @@
         </is>
       </c>
       <c r="D109" t="n">
-        <v>81</v>
+        <v>11</v>
       </c>
       <c r="E109" t="inlineStr">
         <is>
@@ -3073,7 +3073,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>15:54:07</t>
+          <t>17:04:15</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -3087,7 +3087,7 @@
         </is>
       </c>
       <c r="D110" t="n">
-        <v>90</v>
+        <v>20</v>
       </c>
       <c r="E110" t="inlineStr">
         <is>
@@ -3098,21 +3098,21 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>15:54:07</t>
+          <t>17:04:15</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>17:32</t>
+          <t>17:26</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D111" t="n">
-        <v>98</v>
+        <v>22</v>
       </c>
       <c r="E111" t="inlineStr">
         <is>
@@ -3123,21 +3123,21 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>15:54:07</t>
+          <t>17:04:15</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>17:35</t>
+          <t>17:31</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D112" t="n">
-        <v>101</v>
+        <v>27</v>
       </c>
       <c r="E112" t="inlineStr">
         <is>
@@ -3153,16 +3153,16 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>17:37</t>
+          <t>17:32</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D113" t="n">
-        <v>103</v>
+        <v>98</v>
       </c>
       <c r="E113" t="inlineStr">
         <is>
@@ -3173,23 +3173,323 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>15:54:07</t>
+          <t>17:04:15</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
+          <t>17:35</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D114" t="n">
+        <v>31</v>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>17:04:15</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>17:37</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D115" t="n">
+        <v>33</v>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>17:04:15</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
           <t>17:45</t>
         </is>
       </c>
-      <c r="C114" t="inlineStr">
+      <c r="C116" t="inlineStr">
         <is>
           <t>215B_EL PATO</t>
         </is>
       </c>
-      <c r="D114" t="n">
-        <v>111</v>
-      </c>
-      <c r="E114" t="inlineStr">
+      <c r="D116" t="n">
+        <v>41</v>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>17:04:15</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>17:55</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D117" t="n">
+        <v>51</v>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>17:04:15</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>18:04</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D118" t="n">
+        <v>60</v>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>17:04:15</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>18:15</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D119" t="n">
+        <v>71</v>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>17:04:15</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>18:25</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D120" t="n">
+        <v>81</v>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>17:04:15</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>18:27</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D121" t="n">
+        <v>83</v>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>17:04:15</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>18:34</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D122" t="n">
+        <v>90</v>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>17:04:15</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>18:36</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D123" t="n">
+        <v>92</v>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>17:04:15</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>18:44</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D124" t="n">
+        <v>100</v>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>17:04:15</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>18:54</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D125" t="n">
+        <v>110</v>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>17:04:15</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D126" t="n">
+        <v>116</v>
+      </c>
+      <c r="E126" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3206,7 +3506,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E23"/>
+  <dimension ref="A1:E26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3219,14 +3519,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 15:54:07</t>
+          <t>Última actualización: 17:04:15</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 18</t>
+          <t>Total filas: 21</t>
         </is>
       </c>
     </row>
@@ -3660,7 +3960,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>15:54:07</t>
+          <t>17:04:15</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -3674,7 +3974,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>81</v>
+        <v>11</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -3685,7 +3985,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>15:54:07</t>
+          <t>17:04:15</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -3699,9 +3999,84 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>111</v>
+        <v>41</v>
       </c>
       <c r="E23" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>17:04:15</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>17:55</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>51</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>17:04:15</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>18:15</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>71</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>17:04:15</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>116</v>
+      </c>
+      <c r="E26" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3718,7 +4093,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E24"/>
+  <dimension ref="A1:E25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3731,14 +4106,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 15:54:07</t>
+          <t>Última actualización: 17:04:15</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 19</t>
+          <t>Total filas: 20</t>
         </is>
       </c>
     </row>
@@ -4222,7 +4597,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>15:54:07</t>
+          <t>17:04:15</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -4236,9 +4611,34 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>89</v>
+        <v>19</v>
       </c>
       <c r="E24" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>17:04:15</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>18:45</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>101</v>
+      </c>
+      <c r="E25" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 3472
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-06-28.xlsx
+++ b/data/horarios-141-2026-06-28.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E126"/>
+  <dimension ref="A1:E136"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:04:15</t>
+          <t>Última actualización: 18:13:48</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 121</t>
+          <t>Total filas: 131</t>
         </is>
       </c>
     </row>
@@ -883,7 +883,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D22" t="n">
@@ -908,7 +908,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D23" t="n">
@@ -2158,7 +2158,7 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D73" t="n">
@@ -2183,7 +2183,7 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D74" t="n">
@@ -3298,7 +3298,7 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>17:04:15</t>
+          <t>18:13:47</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
@@ -3312,7 +3312,7 @@
         </is>
       </c>
       <c r="D119" t="n">
-        <v>71</v>
+        <v>2</v>
       </c>
       <c r="E119" t="inlineStr">
         <is>
@@ -3323,21 +3323,21 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>17:04:15</t>
+          <t>18:13:47</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>18:25</t>
+          <t>18:21</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D120" t="n">
-        <v>81</v>
+        <v>8</v>
       </c>
       <c r="E120" t="inlineStr">
         <is>
@@ -3348,21 +3348,21 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>17:04:15</t>
+          <t>18:13:47</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>18:27</t>
+          <t>18:24</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D121" t="n">
-        <v>83</v>
+        <v>11</v>
       </c>
       <c r="E121" t="inlineStr">
         <is>
@@ -3378,16 +3378,16 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>18:34</t>
+          <t>18:25</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D122" t="n">
-        <v>90</v>
+        <v>81</v>
       </c>
       <c r="E122" t="inlineStr">
         <is>
@@ -3403,16 +3403,16 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>18:36</t>
+          <t>18:27</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D123" t="n">
-        <v>92</v>
+        <v>83</v>
       </c>
       <c r="E123" t="inlineStr">
         <is>
@@ -3423,21 +3423,21 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>17:04:15</t>
+          <t>18:13:47</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>18:44</t>
+          <t>18:34</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D124" t="n">
-        <v>100</v>
+        <v>21</v>
       </c>
       <c r="E124" t="inlineStr">
         <is>
@@ -3448,21 +3448,21 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>17:04:15</t>
+          <t>18:13:47</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>18:54</t>
+          <t>18:36</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D125" t="n">
-        <v>110</v>
+        <v>23</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
@@ -3473,23 +3473,273 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
+          <t>18:13:47</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>18:44</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D126" t="n">
+        <v>31</v>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>18:13:47</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>18:54</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D127" t="n">
+        <v>41</v>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>18:13:47</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>18:59</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D128" t="n">
+        <v>46</v>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
           <t>17:04:15</t>
         </is>
       </c>
-      <c r="B126" t="inlineStr">
+      <c r="B129" t="inlineStr">
         <is>
           <t>19:00</t>
         </is>
       </c>
-      <c r="C126" t="inlineStr">
+      <c r="C129" t="inlineStr">
         <is>
           <t>215_EL PELIGRO</t>
         </is>
       </c>
-      <c r="D126" t="n">
+      <c r="D129" t="n">
         <v>116</v>
       </c>
-      <c r="E126" t="inlineStr">
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>18:13:47</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>19:04</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D130" t="n">
+        <v>51</v>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>18:13:47</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>19:12</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D131" t="n">
+        <v>59</v>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>18:13:47</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>19:16</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D132" t="n">
+        <v>63</v>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>18:13:47</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>19:16</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D133" t="n">
+        <v>63</v>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>18:13:47</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>19:24</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D134" t="n">
+        <v>71</v>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>18:13:47</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>19:24</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D135" t="n">
+        <v>71</v>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>18:13:47</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>19:50</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>81_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D136" t="n">
+        <v>97</v>
+      </c>
+      <c r="E136" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3506,7 +3756,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E26"/>
+  <dimension ref="A1:E28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3519,14 +3769,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:04:15</t>
+          <t>Última actualización: 18:13:48</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 21</t>
+          <t>Total filas: 23</t>
         </is>
       </c>
     </row>
@@ -4035,7 +4285,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>17:04:15</t>
+          <t>18:13:47</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -4049,7 +4299,7 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>71</v>
+        <v>2</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -4060,23 +4310,73 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
+          <t>18:13:47</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>18:59</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>46</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
           <t>17:04:15</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr">
+      <c r="B27" t="inlineStr">
         <is>
           <t>19:00</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr">
+      <c r="C27" t="inlineStr">
         <is>
           <t>215_EL PELIGRO</t>
         </is>
       </c>
-      <c r="D26" t="n">
+      <c r="D27" t="n">
         <v>116</v>
       </c>
-      <c r="E26" t="inlineStr">
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>18:13:47</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>19:24</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>71</v>
+      </c>
+      <c r="E28" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4093,7 +4393,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E25"/>
+  <dimension ref="A1:E28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4106,14 +4406,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:04:15</t>
+          <t>Última actualización: 18:13:48</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 20</t>
+          <t>Total filas: 23</t>
         </is>
       </c>
     </row>
@@ -4622,23 +4922,98 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
+          <t>18:13:47</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>18:44</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>31</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
           <t>17:04:15</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr">
+      <c r="B26" t="inlineStr">
         <is>
           <t>18:45</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
+      <c r="C26" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D25" t="n">
+      <c r="D26" t="n">
         <v>101</v>
       </c>
-      <c r="E25" t="inlineStr">
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>18:13:47</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>19:14</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>61</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>18:13:47</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>19:46</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>93</v>
+      </c>
+      <c r="E28" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 3473
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-06-28.xlsx
+++ b/data/horarios-141-2026-06-28.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E136"/>
+  <dimension ref="A1:E149"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:13:48</t>
+          <t>Última actualización: 19:15:23</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 131</t>
+          <t>Total filas: 144</t>
         </is>
       </c>
     </row>
@@ -683,7 +683,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -708,7 +708,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D15" t="n">
@@ -3673,21 +3673,21 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>18:13:47</t>
+          <t>19:15:23</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>19:24</t>
+          <t>19:17</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D134" t="n">
-        <v>71</v>
+        <v>2</v>
       </c>
       <c r="E134" t="inlineStr">
         <is>
@@ -3723,23 +3723,348 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>18:13:47</t>
+          <t>19:15:23</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
+          <t>19:24</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D136" t="n">
+        <v>9</v>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>19:15:23</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>19:25</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D137" t="n">
+        <v>10</v>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>19:15:23</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
           <t>19:50</t>
         </is>
       </c>
-      <c r="C136" t="inlineStr">
+      <c r="C138" t="inlineStr">
         <is>
           <t>81_EL PELIGRO</t>
         </is>
       </c>
-      <c r="D136" t="n">
-        <v>97</v>
-      </c>
-      <c r="E136" t="inlineStr">
+      <c r="D138" t="n">
+        <v>35</v>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>19:15:23</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>19:56</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D139" t="n">
+        <v>41</v>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>19:15:23</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>20:01</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D140" t="n">
+        <v>46</v>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>19:15:23</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D141" t="n">
+        <v>60</v>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>19:15:23</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D142" t="n">
+        <v>60</v>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>19:15:23</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>20:36</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D143" t="n">
+        <v>81</v>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>19:15:23</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>20:39</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D144" t="n">
+        <v>84</v>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>19:15:23</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>20:42</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D145" t="n">
+        <v>87</v>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>19:15:23</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>20:42</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D146" t="n">
+        <v>87</v>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>19:15:23</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>20:57</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D147" t="n">
+        <v>102</v>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>19:15:23</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>21:06</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D148" t="n">
+        <v>111</v>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>19:15:23</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>21:07</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D149" t="n">
+        <v>112</v>
+      </c>
+      <c r="E149" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3756,7 +4081,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E28"/>
+  <dimension ref="A1:E31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3769,14 +4094,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:13:48</t>
+          <t>Última actualización: 19:15:23</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 23</t>
+          <t>Total filas: 26</t>
         </is>
       </c>
     </row>
@@ -4377,6 +4702,81 @@
         <v>71</v>
       </c>
       <c r="E28" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>19:15:23</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>19:25</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>10</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>19:15:23</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>60</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>19:15:23</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>20:39</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>84</v>
+      </c>
+      <c r="E31" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4393,7 +4793,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E28"/>
+  <dimension ref="A1:E31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4406,14 +4806,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:13:48</t>
+          <t>Última actualización: 19:15:23</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 23</t>
+          <t>Total filas: 26</t>
         </is>
       </c>
     </row>
@@ -4997,23 +5397,98 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
+          <t>19:15:23</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>19:15</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>0</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
           <t>18:13:47</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr">
+      <c r="B29" t="inlineStr">
         <is>
           <t>19:46</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
+      <c r="C29" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D28" t="n">
+      <c r="D29" t="n">
         <v>93</v>
       </c>
-      <c r="E28" t="inlineStr">
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>19:15:23</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>19:47</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>32</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>19:15:23</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>20:39</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>84</v>
+      </c>
+      <c r="E31" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 3474
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-06-28.xlsx
+++ b/data/horarios-141-2026-06-28.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E149"/>
+  <dimension ref="A1:E159"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:15:23</t>
+          <t>Última actualización: 20:18:38</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 144</t>
+          <t>Total filas: 154</t>
         </is>
       </c>
     </row>
@@ -883,7 +883,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D22" t="n">
@@ -908,7 +908,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D23" t="n">
@@ -2423,7 +2423,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>13:45:34</t>
+          <t>14:49:46</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -2433,11 +2433,11 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D84" t="n">
-        <v>79</v>
+        <v>15</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
@@ -2448,7 +2448,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>14:49:46</t>
+          <t>13:45:34</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -2458,11 +2458,11 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D85" t="n">
-        <v>15</v>
+        <v>79</v>
       </c>
       <c r="E85" t="inlineStr">
         <is>
@@ -3858,7 +3858,7 @@
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D141" t="n">
@@ -3883,7 +3883,7 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D142" t="n">
@@ -3898,21 +3898,21 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>19:15:23</t>
+          <t>20:18:38</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>20:36</t>
+          <t>20:19</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D143" t="n">
-        <v>81</v>
+        <v>1</v>
       </c>
       <c r="E143" t="inlineStr">
         <is>
@@ -3923,21 +3923,21 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>19:15:23</t>
+          <t>20:18:38</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>20:39</t>
+          <t>20:36</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D144" t="n">
-        <v>84</v>
+        <v>18</v>
       </c>
       <c r="E144" t="inlineStr">
         <is>
@@ -3948,21 +3948,21 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>19:15:23</t>
+          <t>20:18:38</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>20:42</t>
+          <t>20:39</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D145" t="n">
-        <v>87</v>
+        <v>21</v>
       </c>
       <c r="E145" t="inlineStr">
         <is>
@@ -3998,21 +3998,21 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>19:15:23</t>
+          <t>20:18:38</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>20:57</t>
+          <t>20:42</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D147" t="n">
-        <v>102</v>
+        <v>24</v>
       </c>
       <c r="E147" t="inlineStr">
         <is>
@@ -4023,21 +4023,21 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>19:15:23</t>
+          <t>20:18:38</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>21:06</t>
+          <t>20:51</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D148" t="n">
-        <v>111</v>
+        <v>33</v>
       </c>
       <c r="E148" t="inlineStr">
         <is>
@@ -4048,23 +4048,273 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
+          <t>20:18:38</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>20:56</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D149" t="n">
+        <v>38</v>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
           <t>19:15:23</t>
         </is>
       </c>
-      <c r="B149" t="inlineStr">
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>20:57</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D150" t="n">
+        <v>102</v>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>20:18:38</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>21:05</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D151" t="n">
+        <v>47</v>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>19:15:23</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>21:06</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D152" t="n">
+        <v>111</v>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>19:15:23</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
         <is>
           <t>21:07</t>
         </is>
       </c>
-      <c r="C149" t="inlineStr">
+      <c r="C153" t="inlineStr">
         <is>
           <t>15_ABASTO</t>
         </is>
       </c>
-      <c r="D149" t="n">
+      <c r="D153" t="n">
         <v>112</v>
       </c>
-      <c r="E149" t="inlineStr">
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>20:18:38</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>21:34</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D154" t="n">
+        <v>76</v>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>20:18:38</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>21:35</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D155" t="n">
+        <v>77</v>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>20:18:38</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>21:37</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
+        </is>
+      </c>
+      <c r="D156" t="n">
+        <v>79</v>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>20:18:38</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>21:38</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D157" t="n">
+        <v>80</v>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>20:18:38</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>21:58</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D158" t="n">
+        <v>100</v>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>20:18:38</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>22:07</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D159" t="n">
+        <v>109</v>
+      </c>
+      <c r="E159" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4094,7 +4344,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:15:23</t>
+          <t>Última actualización: 20:18:38</t>
         </is>
       </c>
     </row>
@@ -4760,7 +5010,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>19:15:23</t>
+          <t>20:18:38</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -4774,7 +5024,7 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>84</v>
+        <v>21</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -4793,7 +5043,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E31"/>
+  <dimension ref="A1:E34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4806,14 +5056,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:15:23</t>
+          <t>Última actualización: 20:18:38</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 26</t>
+          <t>Total filas: 29</t>
         </is>
       </c>
     </row>
@@ -5472,25 +5722,100 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
+          <t>20:18:38</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>20:38</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>20</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
           <t>19:15:23</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr">
+      <c r="B32" t="inlineStr">
         <is>
           <t>20:39</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
+      <c r="C32" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D31" t="n">
+      <c r="D32" t="n">
         <v>84</v>
       </c>
-      <c r="E31" t="inlineStr">
+      <c r="E32" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>20:18:38</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>21:31</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>73</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>20:18:38</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>22:09</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-40 Y 115</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>111</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 3475
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-06-28.xlsx
+++ b/data/horarios-141-2026-06-28.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E159"/>
+  <dimension ref="A1:E167"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:18:38</t>
+          <t>Última actualización: 22:32:42</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 154</t>
+          <t>Total filas: 162</t>
         </is>
       </c>
     </row>
@@ -2158,7 +2158,7 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D73" t="n">
@@ -2183,7 +2183,7 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D74" t="n">
@@ -2423,7 +2423,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>14:49:46</t>
+          <t>13:45:34</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -2433,11 +2433,11 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D84" t="n">
-        <v>15</v>
+        <v>79</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
@@ -2448,7 +2448,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>13:45:34</t>
+          <t>14:49:46</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -2458,11 +2458,11 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D85" t="n">
-        <v>79</v>
+        <v>15</v>
       </c>
       <c r="E85" t="inlineStr">
         <is>
@@ -3698,7 +3698,7 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>18:13:47</t>
+          <t>19:15:23</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
@@ -3708,11 +3708,11 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D135" t="n">
-        <v>71</v>
+        <v>9</v>
       </c>
       <c r="E135" t="inlineStr">
         <is>
@@ -3723,7 +3723,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>19:15:23</t>
+          <t>18:13:47</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
@@ -3733,11 +3733,11 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D136" t="n">
-        <v>9</v>
+        <v>71</v>
       </c>
       <c r="E136" t="inlineStr">
         <is>
@@ -3858,7 +3858,7 @@
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D141" t="n">
@@ -3883,7 +3883,7 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D142" t="n">
@@ -4315,6 +4315,206 @@
         <v>109</v>
       </c>
       <c r="E159" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>22:32:42</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>22:35</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D160" t="n">
+        <v>3</v>
+      </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>22:32:42</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>22:36</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D161" t="n">
+        <v>4</v>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>22:32:42</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>22:43</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D162" t="n">
+        <v>11</v>
+      </c>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>22:32:42</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>22:55</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D163" t="n">
+        <v>23</v>
+      </c>
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>22:32:42</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>23:06</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D164" t="n">
+        <v>34</v>
+      </c>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>22:32:42</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>23:26</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D165" t="n">
+        <v>54</v>
+      </c>
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>22:32:42</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>23:36</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D166" t="n">
+        <v>64</v>
+      </c>
+      <c r="E166" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>22:32:42</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>23:40</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D167" t="n">
+        <v>68</v>
+      </c>
+      <c r="E167" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4331,7 +4531,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E31"/>
+  <dimension ref="A1:E33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4344,14 +4544,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:18:38</t>
+          <t>Última actualización: 22:32:42</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 26</t>
+          <t>Total filas: 28</t>
         </is>
       </c>
     </row>
@@ -5027,6 +5227,56 @@
         <v>21</v>
       </c>
       <c r="E31" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>22:32:42</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>22:36</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>4</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>22:32:42</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>23:40</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>68</v>
+      </c>
+      <c r="E33" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5056,7 +5306,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:18:38</t>
+          <t>Última actualización: 22:32:42</t>
         </is>
       </c>
     </row>

</xml_diff>